<commit_message>
Fix sensitivity analysis — Year 1 locked at 30% ramp across all scenarios
Root cause: base_fcff_s() applied the sensitivity utilisation parameter to
ALL 6 years including Year 1.  At steady-state util ≥ 55%, Year 1 FCFF
turned positive (revenue > CapEx + costs in USD), producing an all-positive
FCF stream with no sign change → IRR solver hit its 50x clamp → every cell
showed ~5,025%.

Fix:
- Year 1 always uses 0.30 (the ramp year) in base_fcff_s()
- Sensitivity parameter (55%–95%) applies only to Years 2–6 (steady-state)
- Added safe_irr() guard that returns None when no sign change exists
- Cell writer checks for nan/None and shows 'n/a' instead of garbage

Verified: Year 1 FCFF = –$22.3M regardless of sensitivity row.
IRR now ranges 290%–513%; NPV ranges $630M–$1,640M (meaningful variation).
Table headers updated to clarify 'Steady-State Util Yr2–6'.

https://claude.ai/code/session_01LaoqAhCxJv5vcVV5Pgy9p8
</commit_message>
<xml_diff>
--- a/72MW_AI_Factory_Project_Finance_Model_USD.xlsx
+++ b/72MW_AI_Factory_Project_Finance_Model_USD.xlsx
@@ -2810,7 +2810,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="58" t="inlineStr">
         <is>
-          <t>X-Axis: EV/EBITDA Exit Multiple  |  Y-Axis: Blended Utilisation  |  Base Case: 77% × 13.5×  (thick blue border)  |  All USD</t>
+          <t>X-Axis: EV/EBITDA Exit Multiple  |  Y-Axis: Steady-State Utilisation Yr2–6  (Year 1 fixed at 30% ramp)  |  Base Case: 77% × 13.5×  |  All USD</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="65" t="inlineStr">
         <is>
-          <t>TABLE A  |  UNLEVERED PROJECT IRR (%)  —  Blended Utilisation vs EV/EBITDA Exit Multiple  (USD)</t>
+          <t>TABLE A  |  UNLEVERED PROJECT IRR (%)  —  Steady-State Utilisation Yr2–6 vs EV/EBITDA Exit Multiple  (Year 1 always 30% ramp  |  USD)</t>
         </is>
       </c>
     </row>
@@ -2934,25 +2934,25 @@
         </is>
       </c>
       <c r="C9" s="69" t="n">
-        <v>50.25</v>
+        <v>2.903114772395583</v>
       </c>
       <c r="D9" s="69" t="n">
-        <v>50.25</v>
+        <v>2.915161312206786</v>
       </c>
       <c r="E9" s="69" t="n">
-        <v>50.25</v>
+        <v>2.92696049175507</v>
       </c>
       <c r="F9" s="69" t="n">
-        <v>50.25</v>
+        <v>2.944221148262429</v>
       </c>
       <c r="G9" s="69" t="n">
-        <v>50.25</v>
+        <v>2.949863304474572</v>
       </c>
       <c r="H9" s="69" t="n">
-        <v>50.25</v>
+        <v>2.960988083703082</v>
       </c>
       <c r="I9" s="69" t="n">
-        <v>50.25</v>
+        <v>2.971907960571589</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -2962,25 +2962,25 @@
         </is>
       </c>
       <c r="C10" s="69" t="n">
-        <v>50.25</v>
+        <v>3.17175100657586</v>
       </c>
       <c r="D10" s="69" t="n">
-        <v>50.25</v>
+        <v>3.182309667704277</v>
       </c>
       <c r="E10" s="69" t="n">
-        <v>50.25</v>
+        <v>3.192686198516078</v>
       </c>
       <c r="F10" s="69" t="n">
-        <v>50.25</v>
+        <v>3.207925522722591</v>
       </c>
       <c r="G10" s="69" t="n">
-        <v>50.25</v>
+        <v>3.212921935172927</v>
       </c>
       <c r="H10" s="69" t="n">
-        <v>50.25</v>
+        <v>3.222794543740713</v>
       </c>
       <c r="I10" s="69" t="n">
-        <v>50.25</v>
+        <v>3.23251190315432</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -2990,25 +2990,25 @@
         </is>
       </c>
       <c r="C11" s="69" t="n">
-        <v>50.25</v>
+        <v>3.442784233072301</v>
       </c>
       <c r="D11" s="69" t="n">
-        <v>50.25</v>
+        <v>3.452037382396522</v>
       </c>
       <c r="E11" s="69" t="n">
-        <v>50.25</v>
+        <v>3.461156534733067</v>
       </c>
       <c r="F11" s="69" t="n">
-        <v>50.25</v>
+        <v>3.474593985270546</v>
       </c>
       <c r="G11" s="69" t="n">
-        <v>50.25</v>
+        <v>3.479010950271083</v>
       </c>
       <c r="H11" s="69" t="n">
-        <v>50.25</v>
+        <v>3.487754665648275</v>
       </c>
       <c r="I11" s="69" t="n">
-        <v>50.25</v>
+        <v>3.496381322644385</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -3018,25 +3018,25 @@
         </is>
       </c>
       <c r="C12" s="69" t="n">
-        <v>50.25</v>
+        <v>3.715847730872786</v>
       </c>
       <c r="D12" s="69" t="n">
-        <v>50.25</v>
+        <v>3.723965304922918</v>
       </c>
       <c r="E12" s="69" t="n">
-        <v>50.25</v>
+        <v>3.731984096049597</v>
       </c>
       <c r="F12" s="69" t="n">
-        <v>50.25</v>
+        <v>3.743833275402885</v>
       </c>
       <c r="G12" s="69" t="n">
-        <v>50.25</v>
+        <v>3.747736621473411</v>
       </c>
       <c r="H12" s="69" t="n">
-        <v>50.25</v>
+        <v>3.755475684406203</v>
       </c>
       <c r="I12" s="69" t="n">
-        <v>50.25</v>
+        <v>3.763126637166029</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -3046,25 +3046,25 @@
         </is>
       </c>
       <c r="C13" s="69" t="n">
-        <v>50.25</v>
+        <v>4.100924371778293</v>
       </c>
       <c r="D13" s="69" t="n">
-        <v>50.25</v>
+        <v>4.107705085230426</v>
       </c>
       <c r="E13" s="69" t="n">
-        <v>50.25</v>
+        <v>4.114420872019721</v>
       </c>
       <c r="F13" s="70" t="n">
-        <v>50.25</v>
+        <v>4.124376048018171</v>
       </c>
       <c r="G13" s="69" t="n">
-        <v>50.25</v>
+        <v>4.127663551191881</v>
       </c>
       <c r="H13" s="69" t="n">
-        <v>50.25</v>
+        <v>4.13419325458861</v>
       </c>
       <c r="I13" s="69" t="n">
-        <v>50.25</v>
+        <v>4.1406636584919</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -3074,25 +3074,25 @@
         </is>
       </c>
       <c r="C14" s="69" t="n">
-        <v>50.25</v>
+        <v>4.26678336010811</v>
       </c>
       <c r="D14" s="69" t="n">
-        <v>50.25</v>
+        <v>4.27307048171967</v>
       </c>
       <c r="E14" s="69" t="n">
-        <v>50.25</v>
+        <v>4.279303179300434</v>
       </c>
       <c r="F14" s="69" t="n">
-        <v>50.25</v>
+        <v>4.288552636601622</v>
       </c>
       <c r="G14" s="69" t="n">
-        <v>50.25</v>
+        <v>4.291609774884231</v>
       </c>
       <c r="H14" s="69" t="n">
-        <v>50.25</v>
+        <v>4.297685818211543</v>
       </c>
       <c r="I14" s="69" t="n">
-        <v>50.25</v>
+        <v>4.303711731383105</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -3102,25 +3102,25 @@
         </is>
       </c>
       <c r="C15" s="69" t="n">
-        <v>50.25</v>
+        <v>4.544126363653384</v>
       </c>
       <c r="D15" s="69" t="n">
-        <v>50.25</v>
+        <v>4.549682425892795</v>
       </c>
       <c r="E15" s="69" t="n">
-        <v>50.25</v>
+        <v>4.55519771600101</v>
       </c>
       <c r="F15" s="69" t="n">
-        <v>50.25</v>
+        <v>4.563395768445679</v>
       </c>
       <c r="G15" s="69" t="n">
-        <v>50.25</v>
+        <v>4.566108831581641</v>
       </c>
       <c r="H15" s="69" t="n">
-        <v>50.25</v>
+        <v>4.571506033465678</v>
       </c>
       <c r="I15" s="69" t="n">
-        <v>50.25</v>
+        <v>4.576865217542368</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -3130,25 +3130,25 @@
         </is>
       </c>
       <c r="C16" s="69" t="n">
-        <v>50.25</v>
+        <v>4.822437768715413</v>
       </c>
       <c r="D16" s="69" t="n">
-        <v>50.25</v>
+        <v>4.827363158451382</v>
       </c>
       <c r="E16" s="69" t="n">
-        <v>50.25</v>
+        <v>4.832257786058809</v>
       </c>
       <c r="F16" s="69" t="n">
-        <v>50.25</v>
+        <v>4.839543056273282</v>
       </c>
       <c r="G16" s="69" t="n">
-        <v>50.25</v>
+        <v>4.841956592203903</v>
       </c>
       <c r="H16" s="69" t="n">
-        <v>50.25</v>
+        <v>4.846761662129653</v>
       </c>
       <c r="I16" s="69" t="n">
-        <v>50.25</v>
+        <v>4.851537753412092</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -3158,31 +3158,31 @@
         </is>
       </c>
       <c r="C17" s="69" t="n">
-        <v>50.25</v>
+        <v>5.101552074188412</v>
       </c>
       <c r="D17" s="69" t="n">
-        <v>50.25</v>
+        <v>5.105932573833285</v>
       </c>
       <c r="E17" s="69" t="n">
-        <v>50.25</v>
+        <v>5.11028969092283</v>
       </c>
       <c r="F17" s="69" t="n">
-        <v>50.25</v>
+        <v>5.116782180491562</v>
       </c>
       <c r="G17" s="69" t="n">
-        <v>50.25</v>
+        <v>5.118934974315445</v>
       </c>
       <c r="H17" s="69" t="n">
-        <v>50.25</v>
+        <v>5.123223723808162</v>
       </c>
       <c r="I17" s="69" t="n">
-        <v>50.25</v>
+        <v>5.127490257465761</v>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="65" t="inlineStr">
         <is>
-          <t>TABLE B  |  PROJECT NPV at WACC 12.5%  (USD Millions)  —  Blended Utilisation vs Exit Multiple</t>
+          <t>TABLE B  |  PROJECT NPV at WACC 12.5%  (USD Millions)  —  Steady-State Utilisation Yr2–6 vs EV/EBITDA Exit Multiple  (Year 1 always 30% ramp  |  USD)</t>
         </is>
       </c>
     </row>
@@ -3235,25 +3235,25 @@
         </is>
       </c>
       <c r="C21" s="71" t="n">
-        <v>658.3829154062687</v>
+        <v>630.2341154062688</v>
       </c>
       <c r="D21" s="71" t="n">
-        <v>704.7631941264169</v>
+        <v>676.6143941264169</v>
       </c>
       <c r="E21" s="71" t="n">
-        <v>751.1434728465653</v>
-      </c>
-      <c r="F21" s="72" t="n">
-        <v>820.7138909267875</v>
+        <v>722.9946728465652</v>
+      </c>
+      <c r="F21" s="71" t="n">
+        <v>792.5650909267875</v>
       </c>
       <c r="G21" s="72" t="n">
-        <v>843.9040302868617</v>
+        <v>815.7552302868617</v>
       </c>
       <c r="H21" s="72" t="n">
-        <v>890.2843090070097</v>
+        <v>862.1355090070098</v>
       </c>
       <c r="I21" s="72" t="n">
-        <v>936.6645877271581</v>
+        <v>908.5157877271581</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -3263,25 +3263,25 @@
         </is>
       </c>
       <c r="C22" s="71" t="n">
-        <v>728.6880612997277</v>
+        <v>694.9095012997277</v>
       </c>
       <c r="D22" s="71" t="n">
-        <v>779.5313640865711</v>
-      </c>
-      <c r="E22" s="72" t="n">
-        <v>830.3746668734144</v>
+        <v>745.7528040865712</v>
+      </c>
+      <c r="E22" s="71" t="n">
+        <v>796.5961068734146</v>
       </c>
       <c r="F22" s="72" t="n">
-        <v>906.6396210536795</v>
+        <v>872.8610610536797</v>
       </c>
       <c r="G22" s="72" t="n">
-        <v>932.0612724471014</v>
+        <v>898.2827124471014</v>
       </c>
       <c r="H22" s="72" t="n">
-        <v>982.9045752339447</v>
+        <v>949.1260152339446</v>
       </c>
       <c r="I22" s="72" t="n">
-        <v>1033.747878020788</v>
+        <v>999.9693180207881</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
@@ -3291,25 +3291,25 @@
         </is>
       </c>
       <c r="C23" s="71" t="n">
-        <v>798.9932071931867</v>
+        <v>759.5848871931867</v>
       </c>
       <c r="D23" s="72" t="n">
-        <v>854.2995340467253</v>
+        <v>814.8912140467253</v>
       </c>
       <c r="E23" s="72" t="n">
-        <v>909.6058609002639</v>
+        <v>870.1975409002639</v>
       </c>
       <c r="F23" s="72" t="n">
-        <v>992.565351180572</v>
+        <v>953.1570311805719</v>
       </c>
       <c r="G23" s="72" t="n">
-        <v>1020.218514607341</v>
+        <v>980.8101946073411</v>
       </c>
       <c r="H23" s="72" t="n">
-        <v>1075.52484146088</v>
+        <v>1036.11652146088</v>
       </c>
       <c r="I23" s="72" t="n">
-        <v>1130.831168314418</v>
+        <v>1091.422848314418</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
@@ -3319,25 +3319,25 @@
         </is>
       </c>
       <c r="C24" s="72" t="n">
-        <v>869.2983530866456</v>
+        <v>824.2602730866456</v>
       </c>
       <c r="D24" s="72" t="n">
-        <v>929.0677040068795</v>
+        <v>884.0296240068794</v>
       </c>
       <c r="E24" s="72" t="n">
-        <v>988.8370549271133</v>
+        <v>943.7989749271132</v>
       </c>
       <c r="F24" s="72" t="n">
-        <v>1078.491081307464</v>
+        <v>1033.453001307464</v>
       </c>
       <c r="G24" s="72" t="n">
-        <v>1108.375756767581</v>
+        <v>1063.337676767581</v>
       </c>
       <c r="H24" s="72" t="n">
-        <v>1168.145107687815</v>
+        <v>1123.107027687815</v>
       </c>
       <c r="I24" s="72" t="n">
-        <v>1227.914458608049</v>
+        <v>1182.876378608049</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
@@ -3347,25 +3347,25 @@
         </is>
       </c>
       <c r="C25" s="72" t="n">
-        <v>967.7255573374882</v>
+        <v>914.8058133374882</v>
       </c>
       <c r="D25" s="72" t="n">
-        <v>1033.743141951095</v>
+        <v>980.8233979510953</v>
       </c>
       <c r="E25" s="72" t="n">
-        <v>1099.760726564703</v>
+        <v>1046.840982564702</v>
       </c>
       <c r="F25" s="73" t="n">
-        <v>1198.787103485113</v>
+        <v>1145.867359485113</v>
       </c>
       <c r="G25" s="72" t="n">
-        <v>1231.795895791917</v>
+        <v>1178.876151791917</v>
       </c>
       <c r="H25" s="72" t="n">
-        <v>1297.813480405524</v>
+        <v>1244.893736405524</v>
       </c>
       <c r="I25" s="72" t="n">
-        <v>1363.831065019131</v>
+        <v>1310.911321019131</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
@@ -3375,25 +3375,25 @@
         </is>
       </c>
       <c r="C26" s="72" t="n">
-        <v>1009.908644873563</v>
+        <v>953.6110448735633</v>
       </c>
       <c r="D26" s="72" t="n">
-        <v>1078.604043927188</v>
+        <v>1022.306443927188</v>
       </c>
       <c r="E26" s="72" t="n">
-        <v>1147.299442980812</v>
+        <v>1091.001842980812</v>
       </c>
       <c r="F26" s="72" t="n">
-        <v>1250.342541561248</v>
+        <v>1194.044941561248</v>
       </c>
       <c r="G26" s="72" t="n">
-        <v>1284.69024108806</v>
+        <v>1228.39264108806</v>
       </c>
       <c r="H26" s="72" t="n">
-        <v>1353.385640141685</v>
+        <v>1297.088040141685</v>
       </c>
       <c r="I26" s="72" t="n">
-        <v>1422.081039195309</v>
+        <v>1365.783439195309</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -3403,25 +3403,25 @@
         </is>
       </c>
       <c r="C27" s="72" t="n">
-        <v>1080.213790767022</v>
+        <v>1018.286430767022</v>
       </c>
       <c r="D27" s="72" t="n">
-        <v>1153.372213887342</v>
+        <v>1091.444853887342</v>
       </c>
       <c r="E27" s="72" t="n">
-        <v>1226.530637007661</v>
+        <v>1164.603277007661</v>
       </c>
       <c r="F27" s="72" t="n">
-        <v>1336.268271688141</v>
+        <v>1274.340911688141</v>
       </c>
       <c r="G27" s="72" t="n">
-        <v>1372.8474832483</v>
+        <v>1310.9201232483</v>
       </c>
       <c r="H27" s="72" t="n">
-        <v>1446.00590636862</v>
+        <v>1384.07854636862</v>
       </c>
       <c r="I27" s="72" t="n">
-        <v>1519.164329488939</v>
+        <v>1457.236969488939</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
@@ -3431,25 +3431,25 @@
         </is>
       </c>
       <c r="C28" s="72" t="n">
-        <v>1150.518936660481</v>
+        <v>1082.961816660481</v>
       </c>
       <c r="D28" s="72" t="n">
-        <v>1228.140383847496</v>
+        <v>1160.583263847496</v>
       </c>
       <c r="E28" s="72" t="n">
-        <v>1305.761831034511</v>
+        <v>1238.204711034511</v>
       </c>
       <c r="F28" s="72" t="n">
-        <v>1422.194001815032</v>
+        <v>1354.636881815033</v>
       </c>
       <c r="G28" s="72" t="n">
-        <v>1461.00472540854</v>
+        <v>1393.44760540854</v>
       </c>
       <c r="H28" s="72" t="n">
-        <v>1538.626172595555</v>
+        <v>1471.069052595555</v>
       </c>
       <c r="I28" s="72" t="n">
-        <v>1616.247619782569</v>
+        <v>1548.690499782569</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
@@ -3459,25 +3459,25 @@
         </is>
       </c>
       <c r="C29" s="72" t="n">
-        <v>1220.82408255394</v>
+        <v>1147.63720255394</v>
       </c>
       <c r="D29" s="72" t="n">
-        <v>1302.90855380765</v>
+        <v>1229.72167380765</v>
       </c>
       <c r="E29" s="72" t="n">
-        <v>1384.99302506136</v>
+        <v>1311.80614506136</v>
       </c>
       <c r="F29" s="72" t="n">
-        <v>1508.119731941925</v>
+        <v>1434.932851941925</v>
       </c>
       <c r="G29" s="72" t="n">
-        <v>1549.16196756878</v>
+        <v>1475.97508756878</v>
       </c>
       <c r="H29" s="72" t="n">
-        <v>1631.24643882249</v>
+        <v>1558.05955882249</v>
       </c>
       <c r="I29" s="72" t="n">
-        <v>1713.3309100762</v>
+        <v>1640.1440300762</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Remove all AUD references — model is pure USD throughout
Stripped every mention of AUD, AUD/USD FX rate (0.65), and
AUD-to-USD conversion notes from build_model.py, test_model.py,
and the generated Excel workbook. All costs, narratives, cell
labels, block headers, input rows, sensitivity footnotes, and
the waterfall summary row now reference USD only.

Replaced the AUD/FX sensitivity footnote on Sheet 4 with a
power-rate sensitivity note. Removed the AUD/USD exchange rate
input row from Sheet 2 Block 0. Replaced AUD conversion checks
in the test suite with USD-native assertions. All 162 tests pass.

https://claude.ai/code/session_01LaoqAhCxJv5vcVV5Pgy9p8
</commit_message>
<xml_diff>
--- a/72MW_AI_Factory_Project_Finance_Model_USD.xlsx
+++ b/72MW_AI_Factory_Project_Finance_Model_USD.xlsx
@@ -547,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -582,10 +582,10 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="9" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="9" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -789,9 +789,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1176,7 +1173,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Isolated SPV / Project Co  ·  'Project Developer Co'  ×  'Technology Provider'  ·  All figures in USD  ·  AUD/USD: 0.65  ·  June 2026</t>
+          <t>Isolated SPV / Project Co  ·  'Project Developer Co'  ×  'Technology Provider'  ·  All figures in USD  ·  June 2026</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1191,7 @@
           <t>This workbook constructs a standalone Project Finance / SPV model for a 72MW high-performance AI computing infrastructure deployment in the Asia-Pacific region.  All items are isolated from parent-company corporate overhead, legacy assets, and consolidated SG&amp;A.
 'Project Developer Co' — the sovereign AI data-centre operator building and operating the 72MW APAC footprint.
 'Technology Provider'  — the leading silicon vendor supplying 40,000 next-gen GPU clusters under a 6-year credit-support and revenue-sharing agreement.
-CURRENCY NOTE: All figures are denominated in USD.  Cost-side inputs (power, maintenance, CapEx, debt facility) have been converted from AUD source data using an AUD/USD rate of 0.65.  GPU billing revenue is quoted directly in USD as GPU cloud pricing is USD-denominated in the global wholesale market.</t>
+CURRENCY NOTE: All figures are denominated in USD.  GPU billing revenue is quoted directly in USD as GPU cloud pricing is USD-denominated in the global wholesale market.  All cost-side inputs (power, maintenance, CapEx, debt facility) are expressed in USD.</t>
         </is>
       </c>
       <c r="B5" s="6" t="n"/>
@@ -1215,7 +1212,7 @@
 Duration:         6-year strategic collaboration.
 Financing:        Capital-light — Technology Provider funds hardware on credit in exchange for 25% of gross cloud billing revenue, eliminating the traditional ~$260M+ upfront GPU CapEx (in USD terms).
 Pre-Contracted:   77% of portfolio (~55.44MW) secured under multi-year take-or-pay enterprise agreements.
-Project Debt:     $32M USD senior facility at 6.5% p.a. funds fit-out and liquid-cooling infrastructure.</t>
+Project Debt:     $43M USD senior facility ($20M Y1 + $7M Y2 + $16M Y4 re-draw) at 6.5% p.a.; funds fit-out, commissioning, and mid-cycle GPU refresh.</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
@@ -1223,7 +1220,7 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>CURRENCY &amp; FX INPUTS</t>
+          <t>CURRENCY NOTE</t>
         </is>
       </c>
       <c r="B10" s="4" t="n"/>
@@ -1231,16 +1228,16 @@
     <row r="11" ht="190" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>AUD/USD Exchange Rate Applied:  0.65
+          <t>All figures in this model are denominated in USD.
 REVENUE (USD-denominated at source):
-  GPU billing rate: $0.80 USD/GPU-hour — this is the wholesale bulk enterprise rate quoted in USD.  The $2.15/kWh figure in the deal narrative is an effective yield metric, NOT the billing mechanism.
-COSTS (converted from AUD at 0.65):
-  Wholesale power: AUD $0.095/kWh → USD $0.065/kWh
-  Year 1 maintenance: AUD $2.5M → USD $2.5M  (AUD $4.0M × 0.65 ≈ $2.5M)
-  Year 2+ maintenance: AUD $8.5M → USD $5.5M  (AUD $8.5M × 0.65 ≈ $5.5M)
-  Year 1 CapEx: AUD $95M → USD $62M  (AUD $95M × 0.65 ≈ $62M)
-  Mid-cycle refresh CapEx: AUD $45M → USD $30M
-  Project debt facility: AUD $50M → USD $32M</t>
+  GPU billing rate: $0.80 USD/GPU-hour — wholesale bulk enterprise rate quoted in USD.  The $2.15/kWh figure in the deal narrative is an effective yield metric, NOT the billing mechanism.
+COSTS (all USD):
+  Wholesale power: $0.065 USD/kWh
+  Year 1 maintenance: $2.5M USD
+  Year 2+ maintenance: $5.5M USD p.a.
+  Year 1 CapEx: $62M USD — data-centre shell, liquid-cooling, substations
+  Mid-cycle refresh CapEx (Year 4): $30M USD
+  Project debt facility: $43M USD total draws</t>
         </is>
       </c>
       <c r="B11" s="6" t="n"/>
@@ -1370,15 +1367,14 @@
       </c>
       <c r="B28" s="4" t="n"/>
     </row>
-    <row r="29" ht="100" customHeight="1">
+    <row r="29" ht="85" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>1. FX RISK:  Revenue is USD; Australian operating costs are AUD.  FX exposure is a real risk.    Add a natural hedge via USD-denominated power purchase agreements where possible.
-2. POWER ESCALATION:  $0.065/kWh USD base rate (2026).  Add CPI escalation toggle for multi-year sensitivity.
-3. GPU REFRESH:  Year 4 $30M USD assumes partial mid-cycle upgrade.  Earlier successor architecture    launches would front-load this into Year 3.
-4. REV-SHARE:  25% is a modelled estimate.  Bracket at 20/25/30% in sensitivity.
-5. TAX:  30% Australian corporate rate at SPV level.  Transfer pricing on the USD-denominated    revenue-share may trigger additional ATO scrutiny — engage local counsel.
-6. WACC:  12.5% reflects single-asset concentration premium.  May compress if sovereign guarantees obtained.</t>
+          <t>1. POWER ESCALATION:  $0.065/kWh USD base rate (2026).  Add CPI escalation toggle for multi-year sensitivity.
+2. GPU REFRESH:  Year 4 $30M USD assumes partial mid-cycle upgrade.  Earlier successor architecture    launches would front-load this into Year 3.
+3. REV-SHARE:  25% is a modelled estimate.  Bracket at 20/25/30% in sensitivity.
+4. TAX:  30% corporate rate applied at SPV level.  Transfer pricing on the USD-denominated    revenue-share may trigger scrutiny — engage local counsel.
+5. WACC:  12.5% reflects single-asset concentration premium.  May compress if sovereign guarantees obtained.</t>
         </is>
       </c>
       <c r="B29" s="6" t="n"/>
@@ -1416,7 +1412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1443,7 +1439,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>BLOCK 0  ·  Currency &amp; FX</t>
+          <t>BLOCK 0  ·  Currency</t>
         </is>
       </c>
       <c r="B4" s="10" t="n"/>
@@ -1468,416 +1464,401 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>AUD / USD Exchange Rate</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>Applied to convert AUD-denominated costs (power, maintenance, CapEx, debt facility) to USD.  Revenue is quoted directly in USD (GPU cloud pricing is USD-denominated globally).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>BLOCK 1  ·  Infrastructure &amp; Capacity</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="4" t="n"/>
+      <c r="B7" s="10" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Project MW Capacity</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>72</v>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Physical design ceiling of the data-centre envelope — fixed for 6-year term.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Project MW Capacity</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="n">
-        <v>72</v>
+          <t>Hardware Clusters (GPU units)</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>40000</v>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Physical design ceiling of the data-centre envelope — fixed for 6-year term.</t>
+          <t>Next-gen AI server clusters deployed under Technology Provider agreement.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Hardware Clusters (GPU units)</t>
+          <t>Power Density per Cluster (kW/GPU)</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>40000</v>
+        <v>1.8</v>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Next-gen AI server clusters deployed under Technology Provider agreement.</t>
+          <t>Design check: 72,000 kW ÷ 40,000 = 1.8 kW incl. networking + liquid-cooling overhead.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Power Density per Cluster (kW/GPU)</t>
+          <t>Contract Duration (Years)</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1.8</v>
+        <v>6</v>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Design check: 72,000 kW ÷ 40,000 = 1.8 kW incl. networking + liquid-cooling overhead.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Contract Duration (Years)</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
           <t>Strategic collaboration term — aligns hardware refresh cycles with exit horizon.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>BLOCK 2  ·  Revenue &amp; Billing Parameters  (USD)</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="4" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="4" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>GPU Billing Rate (USD / GPU-hour)</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Wholesale bulk enterprise rate in USD.  Significant discount to AWS/Azure spot ($2–4/GPU-hr).  NOTE: $2.15/kWh cited in deal narrative = effective yield metric, NOT the billing formula.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>GPU Billing Rate (USD / GPU-hour)</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="n">
-        <v>0.8</v>
+          <t>Year 1 Blended Utilisation (%)</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>0.3</v>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Wholesale bulk enterprise rate in USD.  Significant discount to AWS/Azure spot ($2–4/GPU-hr).  NOTE: $2.15/kWh cited in deal narrative = effective yield metric, NOT the billing formula.</t>
+          <t>Ramp year — contracted tranche partial, uncontracted minimal.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Year 1 Blended Utilisation (%)</t>
+          <t>Year 2–3 Blended Utilisation (%)</t>
         </is>
       </c>
       <c r="C16" s="17" t="n">
-        <v>0.3</v>
+        <v>0.77</v>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Ramp year — contracted tranche partial, uncontracted minimal.</t>
+          <t>Contracted floor activates.  Take-or-pay agreements enforce billing on ~55.44MW.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Year 2–3 Blended Utilisation (%)</t>
+          <t>Year 4–6 Blended Utilisation (%)</t>
         </is>
       </c>
       <c r="C17" s="17" t="n">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Contracted floor activates.  Take-or-pay agreements enforce billing on ~55.44MW.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>Year 4–6 Blended Utilisation (%)</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
           <t>Steady-state: contracted floor + maturing merchant pipeline adds ~3% uplift.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>BLOCK 3  ·  Cost Parameters  (USD, converted from AUD at 0.65)</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="4" t="n"/>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>BLOCK 3  ·  Cost Parameters  (USD)</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="4" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Technology Provider Revenue Share (%)</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>% of Gross Revenue to chip vendor in lieu of ~$260M USD upfront GPU CapEx.  Bracket at 20–30%.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Technology Provider Revenue Share (%)</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="n">
-        <v>0.25</v>
+          <t>Wholesale Power Rate (USD / kWh)</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>0.065</v>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>% of Gross Revenue to chip vendor in lieu of ~$260M USD upfront GPU CapEx.  Bracket at 20–30%.</t>
+          <t>$0.065 USD/kWh.  Applied to IT load = GPU × 1.8kW × utilisation / PUE(1.4).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Wholesale Power Rate (USD / kWh)</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="n">
-        <v>0.065</v>
+          <t>PUE — Power Usage Effectiveness</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>1.4</v>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>AUD $0.095/kWh × 0.65 = USD $0.065/kWh.  Applied to IT load = GPU × 1.8kW × utilisation / PUE(1.4).</t>
+          <t>1.4 standard for liquid-cooled hyperscale.  Total facility power ÷ PUE = IT load.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>PUE — Power Usage Effectiveness</t>
-        </is>
-      </c>
-      <c r="C23" s="19" t="n">
-        <v>1.4</v>
+          <t>Year 1 Facility Maintenance (USD)</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="n">
+        <v>2500000</v>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>1.4 standard for liquid-cooled hyperscale.  Total facility power ÷ PUE = IT load.</t>
+          <t>$2.5M USD.  Commissioning phase; ramps to $5.5M from Year 2.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Year 1 Facility Maintenance (USD)</t>
+          <t>Year 2+ Facility Maintenance (USD)</t>
         </is>
       </c>
       <c r="C24" s="20" t="n">
-        <v>2500000</v>
+        <v>5500000</v>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>AUD $4.0M × 0.65 ≈ USD $2.5M.  Commissioning phase; ramps to $5.5M from Year 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Year 2+ Facility Maintenance (USD)</t>
-        </is>
-      </c>
-      <c r="C25" s="20" t="n">
-        <v>5500000</v>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>AUD $8.5M × 0.65 ≈ USD $5.5M.  Full operations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+          <t>$5.5M USD p.a.  Full operations — engineers, cooling upkeep, monitoring, security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>BLOCK 4  ·  Capital Structure  (USD)</t>
         </is>
       </c>
-      <c r="B27" s="10" t="n"/>
-      <c r="C27" s="10" t="n"/>
-      <c r="D27" s="10" t="n"/>
-      <c r="E27" s="4" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="4" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Year 1 Project Debt Draw (USD)</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>$20M — set below Year 1 FCFF shortfall ($22.3M) so equity sponsor must fund the gap.  Gives a finite, meaningful Levered IRR.  Equity outlay Year 1 ≈ –$3.6M USD.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Year 1 Project Debt Draw (USD)</t>
+          <t>Year 2 Additional Draw (USD)</t>
         </is>
       </c>
       <c r="C28" s="20" t="n">
-        <v>20000000</v>
+        <v>7000000</v>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>$20M — set below Year 1 FCFF shortfall ($22.3M) so equity sponsor must fund the gap.  Gives a finite, meaningful Levered IRR.  Equity outlay Year 1 ≈ –$3.6M USD.</t>
+          <t>$7M — Phase 2 hardware commissioning draw.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Year 2 Additional Draw (USD)</t>
+          <t>Year 4 Re-draw (USD)</t>
         </is>
       </c>
       <c r="C29" s="20" t="n">
-        <v>7000000</v>
+        <v>16000000</v>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>$7M — Phase 2 hardware commissioning draw.</t>
+          <t>$16M — partially funds $30M mid-cycle GPU refresh CapEx.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Year 4 Re-draw (USD)</t>
-        </is>
-      </c>
-      <c r="C30" s="20" t="n">
-        <v>16000000</v>
+          <t>Project Debt Interest Rate (%)</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="n">
+        <v>0.065</v>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>$16M — partially funds $30M mid-cycle GPU refresh CapEx.</t>
+          <t>Senior secured rate on isolated project facility.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Project Debt Interest Rate (%)</t>
+          <t>Corporate Tax Rate (%)</t>
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>0.065</v>
+        <v>0.3</v>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Senior secured rate on isolated project facility.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Corporate Tax Rate (%)</t>
-        </is>
-      </c>
-      <c r="C32" s="17" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E32" s="13" t="inlineStr">
-        <is>
           <t>Australian statutory rate applied at SPV level (30%).</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>BLOCK 5  ·  Valuation &amp; Exit  (USD)</t>
         </is>
       </c>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="4" t="n"/>
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="10" t="n"/>
+      <c r="E33" s="4" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Project WACC (%)</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>Weighted Average Cost of Capital for unlevered DCF discounting.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Project WACC (%)</t>
+          <t>Perpetuity Growth Rate — g (%)</t>
         </is>
       </c>
       <c r="C35" s="17" t="n">
-        <v>0.125</v>
+        <v>0.005</v>
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>Weighted Average Cost of Capital for unlevered DCF discounting.</t>
+          <t>Fixed 72MW ceiling → inflation-only growth assumption.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Perpetuity Growth Rate — g (%)</t>
-        </is>
-      </c>
-      <c r="C36" s="17" t="n">
-        <v>0.005</v>
+          <t>EV/EBITDA — Downside Exit</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="n">
+        <v>10</v>
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>Fixed 72MW ceiling → inflation-only growth assumption.</t>
+          <t>Distressed sale / market de-rating scenario.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>EV/EBITDA — Downside Exit</t>
+          <t>EV/EBITDA — Base Case Exit</t>
         </is>
       </c>
       <c r="C37" s="21" t="n">
-        <v>10</v>
+        <v>13.5</v>
       </c>
       <c r="E37" s="13" t="inlineStr">
         <is>
-          <t>Distressed sale / market de-rating scenario.</t>
+          <t>Negotiated strategic sale — modest discount to APAC peers (14–18×).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>EV/EBITDA — Base Case Exit</t>
+          <t>EV/EBITDA — Upside Exit</t>
         </is>
       </c>
       <c r="C38" s="21" t="n">
-        <v>13.5</v>
+        <v>16</v>
       </c>
       <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>Negotiated strategic sale — modest discount to APAC peers (14–18×).</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>EV/EBITDA — Upside Exit</t>
-        </is>
-      </c>
-      <c r="C39" s="21" t="n">
-        <v>16</v>
-      </c>
-      <c r="E39" s="13" t="inlineStr">
         <is>
           <t>Portfolio sale or SPV IPO capturing sovereign AI infrastructure premium.</t>
         </is>
@@ -1885,14 +1866,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1934,7 +1915,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Project Developer Co  ×  Technology Provider  ·  6-Year Framework  ·  AUD/USD: 0.65</t>
+          <t>Project Developer Co  ×  Technology Provider  ·  6-Year Framework  ·  USD</t>
         </is>
       </c>
       <c r="B2" s="24" t="n"/>
@@ -2088,8 +2069,8 @@
       </c>
       <c r="H8" s="30" t="inlineStr">
         <is>
-          <t>Power cost in USD = GPU_N × 1.8kW × utilisation × 8,760hrs × $0.065/kWh ÷ PUE(1.4).
-AUD $0.095/kWh × 0.65 FX = USD $0.065/kWh.  Tracks utilisation — partially variable with GPU spin-up.</t>
+          <t>Power cost = GPU_N × 1.8kW × utilisation × 8,760hrs × $0.065 USD/kWh ÷ PUE(1.4).
+Partially variable with GPU spin-up — tracks utilisation.</t>
         </is>
       </c>
     </row>
@@ -2119,8 +2100,7 @@
       </c>
       <c r="H9" s="30" t="inlineStr">
         <is>
-          <t>USD figures: AUD source × 0.65 FX rate.
-Year 1: $2.5M (commissioning phase).  Year 2+: $5.5M p.a. (full operations — on-site engineers, cooling upkeep, monitoring, security, facilities management).</t>
+          <t>Year 1: $2.5M USD (commissioning phase).  Year 2+: $5.5M USD p.a. (full operations — on-site engineers, cooling upkeep, monitoring, security, facilities management).</t>
         </is>
       </c>
     </row>
@@ -2180,8 +2160,7 @@
       </c>
       <c r="H11" s="30" t="inlineStr">
         <is>
-          <t>USD figures: AUD source × 0.65 FX.
-  Fit-out $62M / 5yr = $12.4M/yr (Years 1–5)
+          <t xml:space="preserve">  Fit-out $62M USD / 5yr = $12.4M/yr (Years 1–5)
   Hardware tranche 1 / 4yr = $5.7M/yr (Years 1–4)
   Hardware tranche 2 from Yr2 / 4yr = $14.4M/yr (Years 2–5)
 Non-cash — reversed in FCF derivation below.</t>
@@ -2377,8 +2356,7 @@
       </c>
       <c r="H19" s="30" t="inlineStr">
         <is>
-          <t>USD figures (AUD source × 0.65):
-Year 1: –$62M  Fit-out, liquid-cooling manifolds, substations.
+          <t>Year 1: –$62M USD  Fit-out, liquid-cooling manifolds, substations.
 Year 2–3: –$10M  Routine maintenance.
 Year 4: –$30M  Mid-cycle GPU refresh ($16M funded by debt re-draw).
 Year 5–6: –$10M  Tail maintenance.</t>
@@ -3553,12 +3531,12 @@
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="74" t="inlineStr">
         <is>
-          <t>FX Sensitivity</t>
+          <t>Power Rate Sensitivity</t>
         </is>
       </c>
       <c r="C35" s="75" t="inlineStr">
         <is>
-          <t>Revenue is USD; power and maintenance costs are USD (converted from AUD).  If AUD strengthens vs USD (e.g., rate moves from 0.65 to 0.70), cost-side increases by ~7.7% in USD terms while revenue is unaffected — add an FX sensitivity column for completeness.</t>
+          <t>Power cost is $0.065 USD/kWh base.  A 10% increase in the power rate reduces EBITDA by ~$3M p.a. at steady-state utilisation — material but well within EBITDA coverage.  Consider adding a power escalation toggle for multi-year stress testing.</t>
         </is>
       </c>
       <c r="D35" s="76" t="n"/>
@@ -3615,7 +3593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4198,25 +4176,8 @@
       <c r="F28" s="10" t="n"/>
       <c r="G28" s="4" t="n"/>
     </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="74" t="inlineStr">
-        <is>
-          <t>AUD / USD Exchange Rate Applied</t>
-        </is>
-      </c>
-      <c r="B29" s="87" t="inlineStr">
-        <is>
-          <t>0.65</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="4" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="B28:G28"/>
@@ -4225,7 +4186,6 @@
     <mergeCell ref="B27:G27"/>
     <mergeCell ref="B26:G26"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B29:G29"/>
     <mergeCell ref="B25:G25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>